<commit_message>
all in new .odt template
</commit_message>
<xml_diff>
--- a/docs/test runs.xlsx
+++ b/docs/test runs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Amounts" sheetId="1" state="visible" r:id="rId3"/>
@@ -133,6 +133,7 @@
     </font>
     <font>
       <sz val="13"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -144,8 +145,16 @@
     </font>
     <font>
       <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -153,11 +162,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -168,12 +172,19 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -202,7 +213,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -223,8 +234,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -335,8 +362,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Porovnanie modelov podľa WER</a:t>
             </a:r>
@@ -359,9 +390,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="0.476575028636884"/>
-          <c:y val="0.142961219457521"/>
+          <c:y val="0.142905178211163"/>
           <c:w val="0.495189003436426"/>
-          <c:h val="0.711611746245237"/>
+          <c:h val="0.711499663752522"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -541,11 +572,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="76714135"/>
-        <c:axId val="75039707"/>
+        <c:axId val="801057"/>
+        <c:axId val="24557783"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="76714135"/>
+        <c:axId val="801057"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -565,8 +596,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Model</a:t>
                 </a:r>
@@ -608,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75039707"/>
+        <c:crossAx val="24557783"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -616,7 +651,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75039707"/>
+        <c:axId val="24557783"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -645,8 +680,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Priemerný WER</a:t>
                 </a:r>
@@ -688,7 +727,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76714135"/>
+        <c:crossAx val="801057"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -734,8 +773,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Porovnanie modelov podľa CER</a:t>
             </a:r>
@@ -757,10 +800,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.476547734952179"/>
-          <c:y val="0.142889162837611"/>
-          <c:w val="0.495160643720291"/>
-          <c:h val="0.711531995965482"/>
+          <c:x val="0.47651775486827"/>
+          <c:y val="0.142905178211163"/>
+          <c:w val="0.495131729667812"/>
+          <c:h val="0.711499663752522"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -940,11 +983,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="52307051"/>
-        <c:axId val="42555643"/>
+        <c:axId val="91668631"/>
+        <c:axId val="23656894"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="52307051"/>
+        <c:axId val="91668631"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -964,8 +1007,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Model</a:t>
                 </a:r>
@@ -1007,7 +1054,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42555643"/>
+        <c:crossAx val="23656894"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1015,7 +1062,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42555643"/>
+        <c:axId val="23656894"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1045,8 +1092,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Priemerný CER</a:t>
                 </a:r>
@@ -1088,7 +1139,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52307051"/>
+        <c:crossAx val="91668631"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1134,8 +1185,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Rýchlosť prepisu modelov</a:t>
             </a:r>
@@ -1158,9 +1213,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="0.441734090085738"/>
-          <c:y val="0.140777843252799"/>
+          <c:y val="0.140718915733648"/>
           <c:w val="0.492452602342712"/>
-          <c:h val="0.650677666470242"/>
+          <c:h val="0.650559811431939"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -1328,11 +1383,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="35513244"/>
-        <c:axId val="52684829"/>
+        <c:axId val="94962989"/>
+        <c:axId val="14938605"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="35513244"/>
+        <c:axId val="94962989"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1352,8 +1407,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Model</a:t>
                 </a:r>
@@ -1395,7 +1454,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52684829"/>
+        <c:crossAx val="14938605"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1403,7 +1462,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52684829"/>
+        <c:axId val="14938605"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1432,8 +1491,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Sekundy spracovania na 1 sekundu audia</a:t>
                 </a:r>
@@ -1444,8 +1507,8 @@
             <c:manualLayout>
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
-              <c:x val="0.44539032783916"/>
-              <c:y val="0.884869196323356"/>
+              <c:x val="0.445417220142495"/>
+              <c:y val="0.884737772539776"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -1483,7 +1546,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35513244"/>
+        <c:crossAx val="94962989"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1529,8 +1592,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Porovnanie modelov podľa WER a CER</a:t>
             </a:r>
@@ -1541,8 +1608,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.28455843469064"/>
-          <c:y val="0.0163224516988674"/>
+          <c:x val="0.284520598656724"/>
+          <c:y val="0.016435313714603"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -1563,7 +1630,7 @@
           <c:x val="0.441535776614311"/>
           <c:y val="0.118933925596891"/>
           <c:w val="0.370299857210852"/>
-          <c:h val="0.724486396446419"/>
+          <c:h val="0.724375347029428"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -1600,12 +1667,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1634,49 +1706,49 @@
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>huggingface_whisper_large_v3_czech</c:v>
+                  <c:v>whisper_tiny</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>huggingface_whisper_medium_czech</c:v>
+                  <c:v>whisper_base</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>whisper_large</c:v>
+                  <c:v>whisper_small</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>speech_recognition_google</c:v>
+                  <c:v>huggingface_wav2vec2_xlsr_czech</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>huggingface_wav2vec2_xlsr_czech_sammy</c:v>
+                  <c:v>whisper_medium</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>speech_recognition_groq</c:v>
+                  <c:v>faster_whisper_medium_float16_cuda</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>faster_whisper_large_float16_cuda</c:v>
+                  <c:v>speech_recognition_vosk</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>huggingface_wav2vec2_xlsr_53_czech</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>speech_recognition_vosk</c:v>
+                  <c:v>faster_whisper_large_float16_cuda</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>faster_whisper_medium_float16_cuda</c:v>
+                  <c:v>speech_recognition_groq</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>whisper_medium</c:v>
+                  <c:v>huggingface_wav2vec2_xlsr_czech_sammy</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>huggingface_wav2vec2_xlsr_czech</c:v>
+                  <c:v>speech_recognition_google</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>whisper_small</c:v>
+                  <c:v>whisper_large</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>whisper_base</c:v>
+                  <c:v>huggingface_whisper_medium_czech</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>whisper_tiny</c:v>
+                  <c:v>huggingface_whisper_large_v3_czech</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1688,49 +1760,49 @@
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.0441468721692524</c:v>
+                  <c:v>0.908138646571831</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0914443287122927</c:v>
+                  <c:v>0.732145359088816</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.112411016667618</c:v>
+                  <c:v>0.418928020613512</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.119678415800646</c:v>
+                  <c:v>0.395130170015131</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.137222644731534</c:v>
+                  <c:v>0.236012416163012</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.140363740121024</c:v>
+                  <c:v>0.212571002672446</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.157541755617472</c:v>
+                  <c:v>0.174985413000473</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.164664052820296</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.174985413000473</c:v>
+                  <c:v>0.157541755617472</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.212571002672446</c:v>
+                  <c:v>0.140363740121024</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.236012416163012</c:v>
+                  <c:v>0.137222644731534</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.395130170015131</c:v>
+                  <c:v>0.119678415800646</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.418928020613512</c:v>
+                  <c:v>0.112411016667618</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.732145359088816</c:v>
+                  <c:v>0.0914443287122927</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.908138646571831</c:v>
+                  <c:v>0.0441468721692524</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1766,12 +1838,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1800,49 +1877,49 @@
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>huggingface_whisper_large_v3_czech</c:v>
+                  <c:v>whisper_tiny</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>huggingface_whisper_medium_czech</c:v>
+                  <c:v>whisper_base</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>whisper_large</c:v>
+                  <c:v>whisper_small</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>speech_recognition_google</c:v>
+                  <c:v>huggingface_wav2vec2_xlsr_czech</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>huggingface_wav2vec2_xlsr_czech_sammy</c:v>
+                  <c:v>whisper_medium</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>speech_recognition_groq</c:v>
+                  <c:v>faster_whisper_medium_float16_cuda</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>faster_whisper_large_float16_cuda</c:v>
+                  <c:v>speech_recognition_vosk</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>huggingface_wav2vec2_xlsr_53_czech</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>speech_recognition_vosk</c:v>
+                  <c:v>faster_whisper_large_float16_cuda</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>faster_whisper_medium_float16_cuda</c:v>
+                  <c:v>speech_recognition_groq</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>whisper_medium</c:v>
+                  <c:v>huggingface_wav2vec2_xlsr_czech_sammy</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>huggingface_wav2vec2_xlsr_czech</c:v>
+                  <c:v>speech_recognition_google</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>whisper_small</c:v>
+                  <c:v>whisper_large</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>whisper_base</c:v>
+                  <c:v>huggingface_whisper_medium_czech</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>whisper_tiny</c:v>
+                  <c:v>huggingface_whisper_large_v3_czech</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1854,49 +1931,49 @@
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.0108465551141083</c:v>
+                  <c:v>0.396456691370473</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0226342666643933</c:v>
+                  <c:v>0.279014130933508</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0332052892550728</c:v>
+                  <c:v>0.131130033920739</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0460638599643128</c:v>
+                  <c:v>0.083912055247766</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.027455556100141</c:v>
+                  <c:v>0.0711634580873181</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0415494509686245</c:v>
+                  <c:v>0.0599086107996893</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.0463268620757961</c:v>
+                  <c:v>0.0629669593903209</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.034608729144128</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.0629669593903209</c:v>
+                  <c:v>0.0463268620757961</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.0599086107996893</c:v>
+                  <c:v>0.0415494509686245</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.0711634580873181</c:v>
+                  <c:v>0.027455556100141</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.083912055247766</c:v>
+                  <c:v>0.0460638599643128</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.131130033920739</c:v>
+                  <c:v>0.0332052892550728</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.279014130933508</c:v>
+                  <c:v>0.0226342666643933</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.396456691370473</c:v>
+                  <c:v>0.0108465551141083</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1904,11 +1981,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="45937911"/>
-        <c:axId val="9442405"/>
+        <c:axId val="79824178"/>
+        <c:axId val="64841780"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="45937911"/>
+        <c:axId val="79824178"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1928,8 +2005,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>Model</a:t>
                 </a:r>
@@ -1944,7 +2025,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1961,13 +2042,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9442405"/>
+        <c:crossAx val="64841780"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1975,7 +2060,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9442405"/>
+        <c:axId val="64841780"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2004,8 +2089,12 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr sz="900" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:rPr>
                   <a:t>WER a CER</a:t>
                 </a:r>
@@ -2037,13 +2126,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45937911"/>
+        <c:crossAx val="79824178"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2071,8 +2164,12 @@
         <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
+              <a:ea typeface="DejaVu Sans"/>
             </a:defRPr>
           </a:pPr>
         </a:p>
@@ -2103,9 +2200,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>803520</xdr:colOff>
+      <xdr:colOff>803160</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>123840</xdr:rowOff>
+      <xdr:rowOff>123480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2114,7 +2211,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4994640" y="163080"/>
-        <a:ext cx="6285600" cy="3211920"/>
+        <a:ext cx="6285240" cy="3211560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2138,9 +2235,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>803520</xdr:colOff>
+      <xdr:colOff>803160</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>123840</xdr:rowOff>
+      <xdr:rowOff>123480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2149,7 +2246,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4994640" y="163080"/>
-        <a:ext cx="6285600" cy="3211920"/>
+        <a:ext cx="6285240" cy="3211560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2173,9 +2270,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>480960</xdr:colOff>
+      <xdr:colOff>480600</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>128520</xdr:rowOff>
+      <xdr:rowOff>128160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2184,7 +2281,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5485680" y="162720"/>
-        <a:ext cx="5962320" cy="3054600"/>
+        <a:ext cx="5961960" cy="3054240"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2201,16 +2298,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>39960</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>474120</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>548640</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>28800</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>778680</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>152640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2218,8 +2315,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5521320" y="38160"/>
-        <a:ext cx="6807240" cy="3241800"/>
+        <a:off x="7440120" y="0"/>
+        <a:ext cx="6806880" cy="3241440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2800,7 +2897,6 @@
       <c r="B1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="0"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
@@ -2811,7 +2907,6 @@
       <c r="B2" s="4" t="n">
         <v>0.0108465551141083</v>
       </c>
-      <c r="C2" s="0"/>
       <c r="D2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2821,7 +2916,6 @@
       <c r="B3" s="4" t="n">
         <v>0.0226342666643933</v>
       </c>
-      <c r="C3" s="0"/>
       <c r="D3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2831,7 +2925,6 @@
       <c r="B4" s="4" t="n">
         <v>0.027455556100141</v>
       </c>
-      <c r="C4" s="0"/>
       <c r="D4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2841,7 +2934,6 @@
       <c r="B5" s="4" t="n">
         <v>0.0332052892550728</v>
       </c>
-      <c r="C5" s="0"/>
       <c r="D5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2851,7 +2943,6 @@
       <c r="B6" s="4" t="n">
         <v>0.034608729144128</v>
       </c>
-      <c r="C6" s="0"/>
       <c r="D6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,7 +2952,6 @@
       <c r="B7" s="4" t="n">
         <v>0.0415494509686245</v>
       </c>
-      <c r="C7" s="0"/>
       <c r="D7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2871,7 +2961,6 @@
       <c r="B8" s="4" t="n">
         <v>0.0460638599643128</v>
       </c>
-      <c r="C8" s="0"/>
       <c r="D8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2881,7 +2970,6 @@
       <c r="B9" s="3" t="n">
         <v>0.0463268620757961</v>
       </c>
-      <c r="C9" s="0"/>
       <c r="D9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2891,7 +2979,6 @@
       <c r="B10" s="4" t="n">
         <v>0.0599086107996893</v>
       </c>
-      <c r="C10" s="0"/>
       <c r="D10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2901,7 +2988,6 @@
       <c r="B11" s="4" t="n">
         <v>0.0629669593903209</v>
       </c>
-      <c r="C11" s="0"/>
       <c r="D11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2911,7 +2997,6 @@
       <c r="B12" s="4" t="n">
         <v>0.0711634580873181</v>
       </c>
-      <c r="C12" s="0"/>
       <c r="D12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2921,7 +3006,6 @@
       <c r="B13" s="4" t="n">
         <v>0.083912055247766</v>
       </c>
-      <c r="C13" s="0"/>
       <c r="D13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2931,7 +3015,6 @@
       <c r="B14" s="4" t="n">
         <v>0.131130033920739</v>
       </c>
-      <c r="C14" s="0"/>
       <c r="D14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2941,7 +3024,6 @@
       <c r="B15" s="4" t="n">
         <v>0.279014130933508</v>
       </c>
-      <c r="C15" s="0"/>
       <c r="D15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2951,7 +3033,6 @@
       <c r="B16" s="4" t="n">
         <v>0.396456691370473</v>
       </c>
-      <c r="C16" s="0"/>
       <c r="D16" s="4"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -3148,231 +3229,232 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="20.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.908138646571831</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>0.396456691370473</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.0932991636551523</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>0.732145359088816</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>0.279014130933508</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.058864187630119</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.418928020613512</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0.131130033920739</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.0737053906193861</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.395130170015131</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0.083912055247766</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.0441173506620093</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.236012416163012</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0.0711634580873181</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.130435018511475</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.212571002672446</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0.0599086107996893</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.136177451289278</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.174985413000473</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>0.0629669593903209</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.111690524931908</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.164664052820296</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.034608729144128</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.121666608441389</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.157541755617472</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>0.0463268620757961</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.153283050739494</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.140363740121024</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.0415494509686245</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>4.11859599274385</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.137222644731534</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.027455556100141</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.285522869842013</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.119678415800646</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>0.0460638599643128</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.228220963777834</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.112411016667618</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>0.0332052892550728</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>2.13081619568869</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.0914443287122927</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>0.0226342666643933</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.795146019510512</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B16" s="7" t="n">
         <v>0.0441468721692524</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C16" s="7" t="n">
         <v>0.0108465551141083</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D16" s="7" t="n">
         <v>0.256016071870918</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>0.0914443287122927</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>0.0226342666643933</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>0.795146019510512</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>0.112411016667618</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>0.0332052892550728</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>2.13081619568869</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>0.119678415800646</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0.0460638599643128</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>0.228220963777834</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>0.137222644731534</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>0.027455556100141</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0.285522869842013</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>0.140363740121024</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>0.0415494509686245</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>4.11859599274385</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>0.157541755617472</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>0.0463268620757961</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>0.153283050739494</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>0.164664052820296</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>0.034608729144128</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>0.121666608441389</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>0.174985413000473</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>0.0629669593903209</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0.111690524931908</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>0.212571002672446</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>0.0599086107996893</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>0.136177451289278</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>0.236012416163012</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>0.0711634580873181</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>0.130435018511475</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>0.395130170015131</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>0.083912055247766</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>0.0441173506620093</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>0.418928020613512</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>0.131130033920739</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>0.0737053906193861</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>0.732145359088816</v>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>0.279014130933508</v>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>0.058864187630119</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>0.908138646571831</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>0.396456691370473</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>0.0932991636551523</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>